<commit_message>
NPB自動更新(2軍): 2026-08-30 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/raw/2026-08-30/highlights_20260830.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/raw/2026-08-30/highlights_20260830.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7回裏に値千金の同点ホームランを放ち、試合を振り出しに戻す活躍を見せた。</t>
+          <t>7回裏に起死回生の同点ホームランを放ち、試合の流れを大きく変える活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9回裏2死二三塁でサヨナラタイムリー内野安打を放ち、チームを劇的勝利に導いた。</t>
+          <t>9回裏二死二三塁のチャンスでサヨナラタイムリー内野安打を放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>島田 海吏</t>
+          <t>立石 正広</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8回表満塁のチャンスで勝ち越しタイムリーを放ち、チームの勝利に大きく貢献した。</t>
+          <t>8回表に勝ち越しとなる2点タイムリーツーベースを放ち、チームの勝利に大きく貢献した。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>松下 歩叶</t>
+          <t>島田 海吏</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>阪神</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9回表に同点となる犠牲フライを放ち、土壇場で試合を振り出しに戻す粘りを見せた。</t>
+          <t>8回表の満塁のチャンスで勝ち越しタイムリーを放ち、チームを勢いづける一打となった。</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>リチャード</t>
+          <t>ティマ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3回表にレフトスタンドへ同点ホームランを放ち、試合の流れを大きく引き寄せた。</t>
+          <t>9回表に貴重な2点タイムリーを放ち、チームの勝利を決定づける活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>森 駿太</t>
+          <t>井上 絢登</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1回裏にライトスタンドへ2ランホームランを放ち、序盤でチームに大きなリードをもたらした。</t>
+          <t>9回裏に2点タイムリーを放ち、土壇場でチームを同点に引き戻す活躍を見せた。</t>
         </is>
       </c>
     </row>

</xml_diff>